<commit_message>
added evaluate code for baseline model
</commit_message>
<xml_diff>
--- a/asl_experiments_tracker.xlsx
+++ b/asl_experiments_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\idan\FinalProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F8E238-B3C7-47F4-A93A-B867DCAEA780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1EAB66-7CB4-4E59-8A9D-9832FE8E03A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -587,10 +587,18 @@
       <c r="E5" s="7">
         <v>98.18</v>
       </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
+      <c r="F5" s="7">
+        <v>98.28</v>
+      </c>
+      <c r="G5" s="7">
+        <v>98.3</v>
+      </c>
+      <c r="H5" s="7">
+        <v>98.28</v>
+      </c>
+      <c r="I5" s="7">
+        <v>98.28</v>
+      </c>
       <c r="J5" s="8" t="s">
         <v>31</v>
       </c>

</xml_diff>

<commit_message>
added tuned model and tuned model evaluation
</commit_message>
<xml_diff>
--- a/asl_experiments_tracker.xlsx
+++ b/asl_experiments_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\idan\FinalProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F1EAB66-7CB4-4E59-8A9D-9832FE8E03A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621A41F0-2B1C-4195-8637-F9FC17838D6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
   <si>
     <t>Neural Networks Project - Experiment Tracking</t>
   </si>
@@ -67,9 +67,6 @@
     <t>Baseline</t>
   </si>
   <si>
-    <t>cnn_batchnorm.py</t>
-  </si>
-  <si>
     <t>CNN</t>
   </si>
   <si>
@@ -79,9 +76,6 @@
     <t>cnn_dropout.py</t>
   </si>
   <si>
-    <t>+ Dropout</t>
-  </si>
-  <si>
     <t>resnet18_transfer.py</t>
   </si>
   <si>
@@ -116,6 +110,15 @@
   </si>
   <si>
     <t>27m 47s</t>
+  </si>
+  <si>
+    <t>changed lr,bactch size and epochs num</t>
+  </si>
+  <si>
+    <t>tuned_baseline_hyper_para.py</t>
+  </si>
+  <si>
+    <t>hyper parameters</t>
   </si>
 </sst>
 </file>
@@ -495,7 +498,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="2" max="2" width="31.125" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="26" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
@@ -550,7 +553,7 @@
         <v>5</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>6</v>
@@ -600,22 +603,22 @@
         <v>98.28</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="K5" s="9"/>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" ht="28.5">
       <c r="A6" s="5">
         <v>2</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>16</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>17</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
@@ -623,20 +626,22 @@
       <c r="H6" s="7"/>
       <c r="I6" s="7"/>
       <c r="J6" s="8"/>
-      <c r="K6" s="9"/>
+      <c r="K6" s="9" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="5">
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
@@ -651,13 +656,13 @@
         <v>4</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>20</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
@@ -672,13 +677,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
@@ -833,7 +838,7 @@
     </row>
     <row r="22" spans="1:11" ht="15">
       <c r="A22" s="18" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
@@ -851,7 +856,7 @@
         <v>1</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
@@ -868,7 +873,7 @@
         <v>2</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
@@ -885,7 +890,7 @@
         <v>3</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
@@ -902,7 +907,7 @@
         <v>4</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>

</xml_diff>

<commit_message>
added drop out version and evalute to this version
</commit_message>
<xml_diff>
--- a/asl_experiments_tracker.xlsx
+++ b/asl_experiments_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\idan\FinalProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621A41F0-2B1C-4195-8637-F9FC17838D6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{353E5815-A7CF-44E6-AD39-F2ED657EE0DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="36">
   <si>
     <t>Neural Networks Project - Experiment Tracking</t>
   </si>
@@ -58,9 +58,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>baseLine_model.py</t>
-  </si>
-  <si>
     <t>Simple CNN</t>
   </si>
   <si>
@@ -70,12 +67,6 @@
     <t>CNN</t>
   </si>
   <si>
-    <t>+ BatchNorm</t>
-  </si>
-  <si>
-    <t>cnn_dropout.py</t>
-  </si>
-  <si>
     <t>resnet18_transfer.py</t>
   </si>
   <si>
@@ -119,6 +110,24 @@
   </si>
   <si>
     <t>hyper parameters</t>
+  </si>
+  <si>
+    <t>41m 55s</t>
+  </si>
+  <si>
+    <t>return to the baseline hyperparameters, added conv layer and added dropout</t>
+  </si>
+  <si>
+    <t>base_line_model.py</t>
+  </si>
+  <si>
+    <t>improved_cnn_dropout.py</t>
+  </si>
+  <si>
+    <t>another conv layer + Dropout</t>
+  </si>
+  <si>
+    <t>28m 27s</t>
   </si>
 </sst>
 </file>
@@ -553,7 +562,7 @@
         <v>5</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>6</v>
@@ -579,13 +588,13 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
         <v>13</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>14</v>
       </c>
       <c r="E5" s="7">
         <v>98.18</v>
@@ -603,66 +612,92 @@
         <v>98.28</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="K5" s="9"/>
     </row>
-    <row r="6" spans="1:11" ht="28.5">
+    <row r="6" spans="1:11">
       <c r="A6" s="5">
         <v>2</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="8"/>
+        <v>29</v>
+      </c>
+      <c r="E6" s="7">
+        <v>97.53</v>
+      </c>
+      <c r="F6" s="7">
+        <v>97.89</v>
+      </c>
+      <c r="G6" s="7">
+        <v>97.93</v>
+      </c>
+      <c r="H6" s="7">
+        <v>97.89</v>
+      </c>
+      <c r="I6" s="7">
+        <v>97.89</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>30</v>
+      </c>
       <c r="K6" s="9" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="28.5">
       <c r="A7" s="5">
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="9"/>
+        <v>34</v>
+      </c>
+      <c r="E7" s="7">
+        <v>99.72</v>
+      </c>
+      <c r="F7" s="7">
+        <v>99.68</v>
+      </c>
+      <c r="G7" s="7">
+        <v>99.68</v>
+      </c>
+      <c r="H7" s="7">
+        <v>99.68</v>
+      </c>
+      <c r="I7" s="7">
+        <v>99.68</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="5">
         <v>4</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
@@ -677,13 +712,13 @@
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
@@ -838,7 +873,7 @@
     </row>
     <row r="22" spans="1:11" ht="15">
       <c r="A22" s="18" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
@@ -856,7 +891,7 @@
         <v>1</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
@@ -873,7 +908,7 @@
         <v>2</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
@@ -890,7 +925,7 @@
         <v>3</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
@@ -907,7 +942,7 @@
         <v>4</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>

</xml_diff>

<commit_message>
Add VGG16 transfer learning experiment
</commit_message>
<xml_diff>
--- a/asl_experiments_tracker.xlsx
+++ b/asl_experiments_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\idan\FinalProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{353E5815-A7CF-44E6-AD39-F2ED657EE0DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A540A82A-662F-44A6-A8BD-4273D58C2032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
   <si>
     <t>Neural Networks Project - Experiment Tracking</t>
   </si>
@@ -67,12 +67,6 @@
     <t>CNN</t>
   </si>
   <si>
-    <t>resnet18_transfer.py</t>
-  </si>
-  <si>
-    <t>ResNet18</t>
-  </si>
-  <si>
     <t>Transfer Learning</t>
   </si>
   <si>
@@ -128,6 +122,18 @@
   </si>
   <si>
     <t>28m 27s</t>
+  </si>
+  <si>
+    <t>49m 10s</t>
+  </si>
+  <si>
+    <t>VGG16_transfer_learning.py</t>
+  </si>
+  <si>
+    <t>VGG16</t>
+  </si>
+  <si>
+    <t>pre trained model VGG16 on image net</t>
   </si>
 </sst>
 </file>
@@ -562,7 +568,7 @@
         <v>5</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>6</v>
@@ -588,7 +594,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>12</v>
@@ -612,7 +618,7 @@
         <v>98.28</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K5" s="9"/>
     </row>
@@ -621,13 +627,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E6" s="7">
         <v>97.53</v>
@@ -645,10 +651,10 @@
         <v>97.89</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="28.5">
@@ -656,13 +662,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E7" s="7">
         <v>99.72</v>
@@ -680,10 +686,10 @@
         <v>99.68</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -691,34 +697,46 @@
         <v>4</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="9"/>
+        <v>36</v>
+      </c>
+      <c r="D8" s="6"/>
+      <c r="E8" s="7">
+        <v>99.88</v>
+      </c>
+      <c r="F8" s="7">
+        <v>99.89</v>
+      </c>
+      <c r="G8" s="7">
+        <v>99.89</v>
+      </c>
+      <c r="H8" s="7">
+        <v>99.89</v>
+      </c>
+      <c r="I8" s="7">
+        <v>99.89</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="5">
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
@@ -873,7 +891,7 @@
     </row>
     <row r="22" spans="1:11" ht="15">
       <c r="A22" s="18" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
@@ -891,7 +909,7 @@
         <v>1</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
@@ -908,7 +926,7 @@
         <v>2</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
@@ -925,7 +943,7 @@
         <v>3</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
@@ -942,7 +960,7 @@
         <v>4</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>

</xml_diff>

<commit_message>
added dedecated folders for evaluation scripts and models
</commit_message>
<xml_diff>
--- a/asl_experiments_tracker.xlsx
+++ b/asl_experiments_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\idan\FinalProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C000B33-53FC-4A04-832E-58876085AFAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F7DE489-D4C3-4FEF-94F7-0ADB78588DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
   <si>
     <t>Neural Networks Project - Experiment Tracking</t>
   </si>
@@ -67,30 +67,9 @@
     <t>CNN</t>
   </si>
   <si>
-    <t>Transfer Learning</t>
-  </si>
-  <si>
-    <t>efficientnet_b0.py</t>
-  </si>
-  <si>
-    <t>EfficientNet-B0</t>
-  </si>
-  <si>
     <t>Guidelines</t>
   </si>
   <si>
-    <t>Best Val Acc is used to select the best checkpoint during training.</t>
-  </si>
-  <si>
-    <t>Test Acc / Precision / Recall / F1 are filled only after evaluating the saved best model on the test set.</t>
-  </si>
-  <si>
-    <t>Runtime should be the full training time for the script.</t>
-  </si>
-  <si>
-    <t>Use Notes for overfitting observations, failed experiments, or conclusions.</t>
-  </si>
-  <si>
     <t>Best Val Acc (%)(Train)</t>
   </si>
   <si>
@@ -134,6 +113,15 @@
   </si>
   <si>
     <t>pre trained model VGG16 on image net</t>
+  </si>
+  <si>
+    <t>20m 8s</t>
+  </si>
+  <si>
+    <t>base_line_data_augmentation</t>
+  </si>
+  <si>
+    <t>base line model with data augmentation</t>
   </si>
 </sst>
 </file>
@@ -311,18 +299,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -525,7 +513,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27.95" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="16"/>
@@ -540,7 +528,7 @@
       <c r="K1" s="16"/>
     </row>
     <row r="2" spans="1:11" ht="21.95" customHeight="1">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="16"/>
@@ -568,7 +556,7 @@
         <v>5</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>6</v>
@@ -594,7 +582,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>12</v>
@@ -618,7 +606,7 @@
         <v>98.28</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="K5" s="9"/>
     </row>
@@ -627,13 +615,13 @@
         <v>2</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E6" s="7">
         <v>97.53</v>
@@ -651,10 +639,10 @@
         <v>97.89</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="28.5">
@@ -662,13 +650,13 @@
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E7" s="7">
         <v>99.72</v>
@@ -686,10 +674,10 @@
         <v>99.68</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -697,10 +685,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="7">
@@ -719,10 +707,10 @@
         <v>99.89</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -730,21 +718,33 @@
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="9"/>
+        <v>12</v>
+      </c>
+      <c r="D9" s="6"/>
+      <c r="E9" s="7">
+        <v>93.45</v>
+      </c>
+      <c r="F9" s="7">
+        <v>93.45</v>
+      </c>
+      <c r="G9" s="7">
+        <v>93.49</v>
+      </c>
+      <c r="H9" s="7">
+        <v>93.45</v>
+      </c>
+      <c r="I9" s="7">
+        <v>93.44</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="5"/>
@@ -890,8 +890,8 @@
       <c r="K20" s="14"/>
     </row>
     <row r="22" spans="1:11" ht="15">
-      <c r="A22" s="18" t="s">
-        <v>18</v>
+      <c r="A22" s="19" t="s">
+        <v>15</v>
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
@@ -905,12 +905,8 @@
       <c r="K22" s="16"/>
     </row>
     <row r="23" spans="1:11" ht="21.95" customHeight="1">
-      <c r="A23" s="1">
-        <v>1</v>
-      </c>
-      <c r="B23" s="19" t="s">
-        <v>19</v>
-      </c>
+      <c r="A23" s="1"/>
+      <c r="B23" s="15"/>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
       <c r="E23" s="16"/>
@@ -922,12 +918,8 @@
       <c r="K23" s="16"/>
     </row>
     <row r="24" spans="1:11" ht="21.95" customHeight="1">
-      <c r="A24" s="1">
-        <v>2</v>
-      </c>
-      <c r="B24" s="19" t="s">
-        <v>20</v>
-      </c>
+      <c r="A24" s="1"/>
+      <c r="B24" s="15"/>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
       <c r="E24" s="16"/>
@@ -939,12 +931,8 @@
       <c r="K24" s="16"/>
     </row>
     <row r="25" spans="1:11" ht="21.95" customHeight="1">
-      <c r="A25" s="1">
-        <v>3</v>
-      </c>
-      <c r="B25" s="19" t="s">
-        <v>21</v>
-      </c>
+      <c r="A25" s="1"/>
+      <c r="B25" s="15"/>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
@@ -956,12 +944,8 @@
       <c r="K25" s="16"/>
     </row>
     <row r="26" spans="1:11" ht="21.95" customHeight="1">
-      <c r="A26" s="1">
-        <v>4</v>
-      </c>
-      <c r="B26" s="19" t="s">
-        <v>22</v>
-      </c>
+      <c r="A26" s="1"/>
+      <c r="B26" s="15"/>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
       <c r="E26" s="16"/>

</xml_diff>